<commit_message>
Make engine 100% VBA by default (no SQL/ACE dependency)
Per user: entire code in VBA, macros run end to end on just Excel.
- Reports_BuildAll now defaults to pure-VBA aggregation; optional SQL/ACE
  path retained behind USE_SQL=False in modReports.
- Docs updated; dropped the abandoned SQL Server scripts.
- simulate still matches the Rust ledger (7497.5 / 31496.5 / 38854 / balanced).

🤖 Generated with [Claude Code](https://claude.com/claude-code)
</commit_message>
<xml_diff>
--- a/dist/GravityLedger.xlsx
+++ b/dist/GravityLedger.xlsx
@@ -140,7 +140,7 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Click the RUN ALL button (added by Add-Macros.vbs). Macros post the journals + FIFO lots; SQL (ADODB/ACE) builds every report.</t>
+          <t xml:space="preserve">Click the RUN ALL button (added by Add-Macros.vbs). 100% VBA macros, end to end — posts journals + FIFO lots, builds every report, reconciles bank lines. Needs only Excel; no database or add-in.</t>
         </is>
       </c>
     </row>
@@ -242,7 +242,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">macro (procedural posting + FIFO)</t>
+          <t xml:space="preserve">VBA: procedural posting + FIFO</t>
         </is>
       </c>
     </row>
@@ -254,7 +254,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SQL: SUM(amount) per account, JOIN chart of accounts</t>
+          <t xml:space="preserve">VBA: SUM(amount) per account</t>
         </is>
       </c>
     </row>
@@ -266,7 +266,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SQL: GROUP BY entity, exchange, asset over Lots (your 'balances by coin per exchange')</t>
+          <t xml:space="preserve">VBA: group by entity, exchange, asset over Lots (your 'balances by coin per exchange')</t>
         </is>
       </c>
     </row>
@@ -278,7 +278,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SQL: GROUP BY entity, asset over Lots</t>
+          <t xml:space="preserve">VBA: group by entity, asset over Lots</t>
         </is>
       </c>
     </row>
@@ -290,7 +290,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SQL: outstanding LIAB:LOAN per entity</t>
+          <t xml:space="preserve">VBA: outstanding LIAB:LOAN per entity</t>
         </is>
       </c>
     </row>
@@ -302,7 +302,7 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SQL aggregates + IFRS derivation</t>
+          <t xml:space="preserve">VBA aggregates + IFRS derivation</t>
         </is>
       </c>
     </row>
@@ -314,7 +314,7 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">macro: match each BankStatement line to its posted cash journal, then tie out statement vs ledger per entity+ccy</t>
+          <t xml:space="preserve">VBA: match each BankStatement line to its posted cash journal, then tie out statement vs ledger per entity+ccy</t>
         </is>
       </c>
     </row>

</xml_diff>